<commit_message>
Finished Create, started edit
</commit_message>
<xml_diff>
--- a/database/tbl2.xlsx
+++ b/database/tbl2.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yorck\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yorck Zisgen\PycharmProjects\Sandboxbox\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFF34452-554C-4727-BC6A-C0EBA51AE1E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F84F58-72E9-497F-B532-11036F352899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34290" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{2EDA8774-3024-4E0D-AF44-959837F7CBA6}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{2EDA8774-3024-4E0D-AF44-959837F7CBA6}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="37">
   <si>
     <t>Tabelle Prompts</t>
   </si>
@@ -53,21 +54,12 @@
     <t>-</t>
   </si>
   <si>
-    <t>rechtstext</t>
-  </si>
-  <si>
-    <t>systemprompt</t>
-  </si>
-  <si>
     <t>"er hat hierzu folgendes angegeben"</t>
   </si>
   <si>
     <t>"weiterhin hat er folgende dokumenteninhalte bereitgestellt"</t>
   </si>
   <si>
-    <t>aufgabenprompt</t>
-  </si>
-  <si>
     <t>{paragraph}</t>
   </si>
   <si>
@@ -80,9 +72,6 @@
     <t>Tabelle Antworten</t>
   </si>
   <si>
-    <t>Antwort</t>
-  </si>
-  <si>
     <t>table_id</t>
   </si>
   <si>
@@ -98,31 +87,67 @@
     <t>Tabelle Fragen</t>
   </si>
   <si>
-    <t>Fragentext</t>
-  </si>
-  <si>
-    <t>Kurzbezeichnung</t>
-  </si>
-  <si>
     <t>text, not null</t>
   </si>
   <si>
-    <t>Hinweis</t>
-  </si>
-  <si>
-    <t>Startfrage</t>
-  </si>
-  <si>
     <t>boolean</t>
   </si>
   <si>
-    <t>Nachfolger_Ja</t>
-  </si>
-  <si>
-    <t>Nachfolger_Nein</t>
-  </si>
-  <si>
-    <t>Nachfolger_Unsicher</t>
+    <t>Bem</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Bez</t>
+  </si>
+  <si>
+    <t>Initial</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Read, Update, Delete</t>
+  </si>
+  <si>
+    <t>Nav Bar -&gt; Create, Edit/Delete</t>
+  </si>
+  <si>
+    <t>Nav Bar -&gt; zwei Modi</t>
+  </si>
+  <si>
+    <t>Urlaub</t>
+  </si>
+  <si>
+    <t>Marleen</t>
+  </si>
+  <si>
+    <t>Kaeser</t>
+  </si>
+  <si>
+    <t>Paper-Nutzung in Diss</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>DSGVO</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Mail an Krönke</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>Nein</t>
+  </si>
+  <si>
+    <t>Unsicher</t>
   </si>
 </sst>
 </file>
@@ -533,7 +558,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3"/>
     </row>
@@ -547,23 +572,23 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B7" s="3"/>
     </row>
@@ -577,23 +602,23 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>3</v>
@@ -601,7 +626,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>3</v>
@@ -609,7 +634,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>3</v>
@@ -617,7 +642,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>3</v>
@@ -625,15 +650,15 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B18" s="3"/>
     </row>
@@ -647,18 +672,18 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -677,29 +702,29 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -707,10 +732,10 @@
         <v>4</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -718,15 +743,15 @@
         <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>3</v>
@@ -736,4 +761,49 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D905F39-F81D-4426-A745-6B03BF30756C}">
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>